<commit_message>
review: add papers 23-25 (intermittent demand), secondary sources for 15/16/18
Exclude engproc-59-00132 (histopathology, off-topic).
</commit_message>
<xml_diff>
--- a/M5_papers_baseline_gap.xlsx
+++ b/M5_papers_baseline_gap.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ghi chú kiểm tra" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M5 Papers'!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M5 Papers'!$A$1:$M$26</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -231,6 +231,7 @@
     <author>Claude (kiểm tra 29/09/2026)</author>
     <author>Claude (rà soát lần 3 – có PDF bài 01–03)</author>
     <author>Claude (rà soát 29/09/2026 – lần 2)</author>
+    <author>Claude (lần 4)</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0">
@@ -506,11 +507,22 @@
 Lý do sửa: Chỉ có abstract.</t>
       </text>
     </comment>
-    <comment ref="F16" authorId="2" shapeId="0">
+    <comment ref="F16" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dự báo vẫn bị lệch (sau này sửa bằng SBA); không cập nhật khi sản phẩm sắp lỗi thời
-Lý do sửa: Viết lại theo nguồn kiểm chứng được (abstract bài 16).</t>
+Lý do sửa: Viết lại theo nguồn kiểm chứng được (abstract bài 16).
+---
+[Lần 4] Giá trị trước:
+Theo abstract bài 16 (TSB): Croston không cập nhật sau các kỳ nhu cầu bằng 0 nên không phù hợp khi hàng lỗi thời, và bị lệch dương (SBA khắc phục lệch)
+Lý do: Bổ sung nguồn thứ cấp đã đọc toàn văn (bài 23).</t>
+      </text>
+    </comment>
+    <comment ref="D17" authorId="3" shapeId="0">
+      <text>
+        <t>[Lần 4] Giá trị trước:
+Phương pháp TSB: cập nhật xác suất có nhu cầu mỗi kỳ, phản ứng nhanh khi nhu cầu suy giảm
+Lý do: Bổ sung nguồn thứ cấp (bài 23).</t>
       </text>
     </comment>
     <comment ref="E17" authorId="2" shapeId="0">
@@ -541,7 +553,7 @@
 Lý do sửa: Tách rõ nhận định nhóm với nội dung bài.</t>
       </text>
     </comment>
-    <comment ref="D19" authorId="1" shapeId="0">
+    <comment ref="D19" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Phân loại nhu cầu theo ADI (ngưỡng 1,32) và CV² (ngưỡng 0,49): smooth / erratic / intermittent / lumpy
@@ -549,7 +561,11 @@
 ---
 [Lần 3] Giá trị trước:
 Phân loại nhu cầu theo ADI và CV² dựa trên so sánh MSE lý thuyết của EWMA, Croston, SBA (abstract). Ngưỡng ADI &gt; 1,32 (nguồn thứ cấp: bài 12 tr. 10). [Chưa kiểm chứng: ngưỡng CV² = 0,49 và tên 4 nhóm]
-Lý do: Ngưỡng nay kiểm chứng được qua bài 01; con số 0,49/1,32 là giá trị làm tròn hay được trích lại.</t>
+Lý do: Ngưỡng nay kiểm chứng được qua bài 01; con số 0,49/1,32 là giá trị làm tròn hay được trích lại.
+---
+[Lần 4] Giá trị trước:
+Phân loại nhu cầu theo ADI và CV², so sánh MSE lý thuyết của EWMA, Croston, SBA (abstract). Ngưỡng CV² = 0,5 và ADI = 4/3 (nguồn thứ cấp: bài 01, tr. 7–8)
+Lý do: Tên 4 nhóm nay kiểm chứng được qua bài 23; ghi rõ có 2 cách ghi ngưỡng.</t>
       </text>
     </comment>
     <comment ref="E19" authorId="2" shapeId="0">
@@ -884,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1891,7 +1907,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Theo abstract bài 16 (TSB): Croston không cập nhật sau các kỳ nhu cầu bằng 0 nên không phù hợp khi hàng lỗi thời, và bị lệch dương (SBA khắc phục lệch)</t>
+          <t>Croston lệch dương; không cập nhật sau các kỳ bằng 0 nên không hợp với hàng lỗi thời (abstract bài 16); SBA ra đời để sửa lệch (bài 23, tr. 1, 4)</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -1924,7 +1940,7 @@
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>[Nội dung] Chỉ đọc được abstract (bài đóng) — 29/09/2026
+          <t>[Nội dung] Chỉ đọc được abstract (bài đóng) — 29/09/2026 + nguồn thứ cấp đã đọc toàn văn (bài 23)
 [Metadata] ✅ Crossref khớp tên/tác giả/tạp chí/trang; DOI chuyển đúng nhà xuất bản (Taylor &amp; Francis có bước chống bot khi mở tự động)</t>
         </is>
       </c>
@@ -1943,9 +1959,9 @@
           <t>https://doi.org/10.1016/j.ejor.2011.05.018</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Phương pháp TSB: cập nhật xác suất có nhu cầu mỗi kỳ, phản ứng nhanh khi nhu cầu suy giảm</t>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>TSB: cập nhật xác suất xảy ra nhu cầu mỗi kỳ, không lệch (abstract); xác suất giảm dần theo hàm mũ, hợp với sản phẩm cuối vòng đời (bài 23, tr. 2, 4)</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1988,7 +2004,7 @@
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>[Nội dung] Chỉ đọc được abstract — 29/09/2026
+          <t>[Nội dung] Chỉ đọc được abstract — 29/09/2026 + nguồn thứ cấp đã đọc toàn văn (bài 23)
 [Metadata] ✅ Crossref khớp tên/tác giả/tạp chí/trang; DOI chuyển đúng nhà xuất bản</t>
         </is>
       </c>
@@ -2073,7 +2089,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Phân loại nhu cầu theo ADI và CV², so sánh MSE lý thuyết của EWMA, Croston, SBA (abstract). Ngưỡng CV² = 0,5 và ADI = 4/3 (nguồn thứ cấp: bài 01, tr. 7–8)</t>
+          <t>Phân loại theo ADI và CV², so sánh MSE của EWMA, Croston, SBA (abstract). Ngưỡng 4/3 và 0,5 (bài 01, tr. 7–8), hoặc 1,32 và 0,49 kèm tên 4 nhóm Smooth/Intermittent/Erratic/Lumpy (bài 23, tr. 10)</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -2116,7 +2132,7 @@
       </c>
       <c r="M19" s="8" t="inlineStr">
         <is>
-          <t>[Nội dung] Chỉ đọc được abstract — 29/09/2026
+          <t>[Nội dung] Chỉ đọc được abstract — 29/09/2026 + nguồn thứ cấp đã đọc toàn văn (bài 23, bài 01)
 [Metadata] ✅ Crossref khớp tên/tác giả/tạp chí/trang; DOI chuyển đúng nhà xuất bản (Taylor &amp; Francis có bước chống bot khi mở tự động)</t>
         </is>
       </c>
@@ -2377,8 +2393,200 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="70.05" customHeight="1">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>A New Approach to Forecast Intermittent Demand and Stock-Keeping-Unit Level Optimization for Spare Parts Management (Sfiris &amp; Koulouriotis, 2025)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/app152212030</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Họ Croston (Croston, SBA, TSB, …) + phương pháp SK mới; chọn mô hình theo SKU (MCOST); chính sách (R, Q) với lead-time demand NB–Bernoulli (tr. 2, 4, 10–11)</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2.050 SKU phụ tùng ô tô × 104 tuần, không công khai (tr. 14, 27)</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Tác giả nêu (tr. 25): lead time cố định 3 ngày; chưa mô hình lịch/sự kiện; chỉ ngành ô tô, dữ liệu tuần</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Sfiris, Koulouriotis</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Applied Sciences (MDPI) 15(22):12030</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/app152212030</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>AI model / method + Domain</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>★★★ (nguồn thứ cấp cho bài 15, 16, 18)</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="inlineStr">
+        <is>
+          <t>[Nội dung] Đã đọc toàn văn (papers_pdf/applsci-15-12030-v3.pdf) — 29/09/2026
+[Metadata] ✅ Crossref khớp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70.05" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Feature engineering for intermittent demand forecasting: zero-detection and forecast performance across GRU, LSTM, and TCN architectures (El-Meehy, El-Kharbotly &amp; El-Beheiry, 2026)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10845-026-02964-7</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>GRU, LSTM, TCN + 20 chiến lược đặc trưng; đề xuất thước đo Z% và NZ% (abstract)</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>19 chuỗi sản phẩm M5 chọn theo 3 mức ADI (1,32; 1,60; 2,00) (tr. 8)</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Tác giả nêu: chỉ dự báo điểm, không xét dự báo xác suất (tr. 26); chưa xét ADI rất cao (tr. 9). Nhận định nhóm: chỉ 19 chuỗi</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>El-Meehy, El-Kharbotly, El-Beheiry</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Journal of Intelligent Manufacturing (Springer)</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10845-026-02964-7</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>AI model / method + M5</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
+        <is>
+          <t>[Nội dung] Đã đọc toàn văn (papers_pdf/s10845-026-02964-7.pdf) — 29/09/2026
+[Metadata] ✅ Crossref khớp</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70.05" customHeight="1">
+      <c r="A26" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Forecasting Critical Spare Parts Demand in Combined Cycle Power Plant Using Ensemble Learning (Putra &amp; Purnomo, 2026)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/engproc2026143030</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Random Forest vs XGBoost (tinh chỉnh) (abstract)</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu mua/sử dụng phụ tùng 2020–2024 của một nhà máy, theo tháng, chọn mặt hàng có chủ đích (tr. 2)</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không có KPI tồn kho; phải loại kỳ bằng 0 khỏi MAPE (abstract)</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Putra, Purnomo</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Engineering Proceedings (MDPI) 143:30 — kỷ yếu ETLTC 2026</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/engproc2026143030</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>Domain (spare parts)</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>★ (tham khảo phụ)</t>
+        </is>
+      </c>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>[Nội dung] Đã đọc toàn văn (papers_pdf/engproc-143-00030.pdf) — 29/09/2026
+[Metadata] ✅ Crossref khớp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M23"/>
+  <autoFilter ref="A1:M26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
@@ -2424,6 +2632,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -2436,7 +2650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4438,6 +4652,178 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>LẦN 4 (29/09/2026): bổ sung bài 23–25 do người dùng gửi</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Theo abstract bài 16 (TSB): Croston không cập nhật sau các kỳ nhu cầu bằng 0 nên không phù hợp khi hàng lỗi thời, và bị lệch dương (SBA khắc phục lệch)</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Croston lệch dương; không cập nhật sau các kỳ bằng 0 nên không hợp với hàng lỗi thời (abstract bài 16); SBA ra đời để sửa lệch (bài 23, tr. 1, 4)</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 4] Bổ sung nguồn thứ cấp đã đọc toàn văn (bài 23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Model đã dùng</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Phương pháp TSB: cập nhật xác suất có nhu cầu mỗi kỳ, phản ứng nhanh khi nhu cầu suy giảm</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>TSB: cập nhật xác suất xảy ra nhu cầu mỗi kỳ, không lệch (abstract); xác suất giảm dần theo hàm mũ, hợp với sản phẩm cuối vòng đời (bài 23, tr. 2, 4)</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 4] Bổ sung nguồn thứ cấp (bài 23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Model đã dùng</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Phân loại nhu cầu theo ADI và CV², so sánh MSE lý thuyết của EWMA, Croston, SBA (abstract). Ngưỡng CV² = 0,5 và ADI = 4/3 (nguồn thứ cấp: bài 01, tr. 7–8)</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Phân loại theo ADI và CV², so sánh MSE của EWMA, Croston, SBA (abstract). Ngưỡng 4/3 và 0,5 (bài 01, tr. 7–8), hoặc 1,32 và 0,49 kèm tên 4 nhóm Smooth/Intermittent/Erratic/Lumpy (bài 23, tr. 10)</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 4] Tên 4 nhóm nay kiểm chứng được qua bài 23; ghi rõ có 2 cách ghi ngưỡng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>(cả dòng)</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>A New Approach to Forecast Intermittent Demand and Stock-Keeping-Unit Level Optimization for Spare Parts Management (Sfiris &amp; Koulouriotis, 2025)</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Bài người dùng gửi; đã đọc toàn văn; metadata qua Crossref</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>(cả dòng)</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr"/>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Feature engineering for intermittent demand forecasting: zero-detection and forecast performance across GRU, LSTM, and TCN architectures (El-Meehy, El-Kharbotly &amp; El-Beheiry, 2026)</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Bài người dùng gửi; đã đọc toàn văn; metadata qua Crossref</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>(cả dòng)</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Forecasting Critical Spare Parts Demand in Combined Cycle Power Plant Using Ensemble Learning (Putra &amp; Purnomo, 2026)</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Bài người dùng gửi; đã đọc toàn văn; metadata qua Crossref</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>(loại)</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>engproc-59-00132.pdf</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Histopathological Image Analysis Using Deep Learning Framework (Vupulluri &amp; Munagala, 2023)</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>KHÔNG đưa vào: bài ảnh mô bệnh học ung thư vú, không liên quan đề tài</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
review: apply PDF audit fixes to Excel (papers 03, 21, 22, 25)
</commit_message>
<xml_diff>
--- a/M5_papers_baseline_gap.xlsx
+++ b/M5_papers_baseline_gap.xlsx
@@ -230,6 +230,7 @@
   <authors>
     <author>Claude (kiểm tra 29/09/2026)</author>
     <author>Claude (rà soát lần 3 – có PDF bài 01–03)</author>
+    <author>Claude (lần 5 – rà soát bằng PDF)</author>
     <author>Claude (rà soát 29/09/2026 – lần 2)</author>
     <author>Claude (lần 4)</author>
   </authors>
@@ -324,7 +325,7 @@
 Lý do: Bổ sung số liệu tham gia.</t>
       </text>
     </comment>
-    <comment ref="F4" authorId="1" shapeId="0">
+    <comment ref="F4" authorId="2" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Cũng giới hạn phân tích ở top 50 đội; ít đội chia sẻ chi tiết mô hình sử dụng
@@ -332,7 +333,11 @@
 ---
 [Lần 3] Giá trị trước:
 [Chưa kiểm chứng — cần mở toàn văn] Ghi chú cũ: giới hạn phân tích ở top 50 đội
-Lý do: Ghi chú 'top 50' ban đầu nằm ở bài Accuracy; bài này nói LightGBM được đại đa số top 50 dùng (tr. 19).</t>
+Lý do: Ghi chú 'top 50' ban đầu nằm ở bài Accuracy; bài này nói LightGBM được đại đa số top 50 dùng (tr. 19).
+---
+[Lần 5] Giá trị trước:
+Nhận định nhóm: không đánh giá việc dùng phân vị cho quyết định tồn kho
+Lý do: Thay nhận định nhóm bằng câu có trong bài (PDF).</t>
       </text>
     </comment>
     <comment ref="B5" authorId="0" shapeId="0">
@@ -412,7 +417,7 @@
 Lý do sửa: Bổ sung tác giả và venue: arXiv ghi 'ICLR 2026'.</t>
       </text>
     </comment>
-    <comment ref="F11" authorId="2" shapeId="0">
+    <comment ref="F11" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 M5 không có ground-truth counterfactual nên chỉ dùng để đánh giá khả năng sinh chuỗi có điều kiện, không đánh giá được tính đúng đắn nhân quả thực sự
@@ -461,7 +466,7 @@
 Lý do sửa: Bổ sung quy mô dữ liệu theo abstract.</t>
       </text>
     </comment>
-    <comment ref="F13" authorId="2" shapeId="0">
+    <comment ref="F13" authorId="3" shapeId="0">
       <text>
         <t>Giá trị cũ:
 Bài chỉ ra hiện chưa có kiến trúc global model chuẩn cho intermittent demand — vẫn là bài toán mở
@@ -486,28 +491,28 @@
 Lý do sửa: Mô tả cũ ('so sánh với ETS') chưa đúng: theo PDF, ETS là mô hình dùng BÊN TRONG e2eTD để dự báo các chuỗi tổng hợp được chọn.</t>
       </text>
     </comment>
-    <comment ref="D15" authorId="2" shapeId="0">
+    <comment ref="D15" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 LightGBM — GBDT với GOSS và EFB, tăng trưởng cây theo lá; hỗ trợ loss Tweedie và quantile
 Lý do sửa: Tách tính năng thư viện khỏi nội dung bài báo.</t>
       </text>
     </comment>
-    <comment ref="E15" authorId="2" shapeId="0">
+    <comment ref="E15" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Nhiều dataset công khai lớn (không phải chuỗi thời gian)
 Lý do sửa: Cụ thể hóa theo toàn văn.</t>
       </text>
     </comment>
-    <comment ref="E16" authorId="2" shapeId="0">
+    <comment ref="E16" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Phân tích lý thuyết / dữ liệu tồn kho
 Lý do sửa: Chỉ có abstract.</t>
       </text>
     </comment>
-    <comment ref="F16" authorId="3" shapeId="0">
+    <comment ref="F16" authorId="4" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dự báo vẫn bị lệch (sau này sửa bằng SBA); không cập nhật khi sản phẩm sắp lỗi thời
@@ -518,42 +523,42 @@
 Lý do: Bổ sung nguồn thứ cấp đã đọc toàn văn (bài 23).</t>
       </text>
     </comment>
-    <comment ref="D17" authorId="3" shapeId="0">
+    <comment ref="D17" authorId="4" shapeId="0">
       <text>
         <t>[Lần 4] Giá trị trước:
 Phương pháp TSB: cập nhật xác suất có nhu cầu mỗi kỳ, phản ứng nhanh khi nhu cầu suy giảm
 Lý do: Bổ sung nguồn thứ cấp (bài 23).</t>
       </text>
     </comment>
-    <comment ref="E17" authorId="2" shapeId="0">
+    <comment ref="E17" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dữ liệu mô phỏng và thực tế
 Lý do sửa: SAI trước đó: ghi 'mô phỏng và thực tế'. Abstract chỉ nêu 'extensive simulation experiment'.</t>
       </text>
     </comment>
-    <comment ref="F17" authorId="2" shapeId="0">
+    <comment ref="F17" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Mô hình thống kê cục bộ, không dùng biến ngoại sinh (giá, sự kiện)
 Lý do sửa: Đồng bộ với E16.</t>
       </text>
     </comment>
-    <comment ref="E18" authorId="2" shapeId="0">
+    <comment ref="E18" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dữ liệu bán lẻ Amazon, điện năng, giao thông
 Lý do sửa: Bổ sung đầy đủ theo toàn văn (trước đó thiếu dataset parts).</t>
       </text>
     </comment>
-    <comment ref="F18" authorId="2" shapeId="0">
+    <comment ref="F18" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Cần GPU và tinh chỉnh siêu tham số; khó diễn giải
 Lý do sửa: Tách rõ nhận định nhóm với nội dung bài.</t>
       </text>
     </comment>
-    <comment ref="D19" authorId="3" shapeId="0">
+    <comment ref="D19" authorId="4" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Phân loại nhu cầu theo ADI (ngưỡng 1,32) và CV² (ngưỡng 0,49): smooth / erratic / intermittent / lumpy
@@ -568,7 +573,7 @@
 Lý do: Tên 4 nhóm nay kiểm chứng được qua bài 23; ghi rõ có 2 cách ghi ngưỡng.</t>
       </text>
     </comment>
-    <comment ref="E19" authorId="2" shapeId="0">
+    <comment ref="E19" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Phân tích lý thuyết + dữ liệu thực
@@ -586,25 +591,53 @@
 Lý do: Bổ sung nguồn.</t>
       </text>
     </comment>
-    <comment ref="D20" authorId="2" shapeId="0">
+    <comment ref="D20" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Tối ưu / chọn mô hình dự báo theo tiêu chí gắn với tồn kho thay vì chỉ sai số dự báo
 Lý do sửa: Toàn văn chưa tải được; 'họ exponential smoothing' chưa kiểm chứng.</t>
       </text>
     </comment>
-    <comment ref="E20" authorId="2" shapeId="0">
+    <comment ref="E20" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dữ liệu bán lẻ và mô phỏng
 Lý do sửa: SAI trước đó: 'bán lẻ và mô phỏng' chưa kiểm chứng.</t>
       </text>
     </comment>
-    <comment ref="F20" authorId="2" shapeId="0">
+    <comment ref="F20" authorId="3" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Chỉ xét mô hình thống kê (họ exponential smoothing), chưa xét mô hình ML toàn cục
 Lý do sửa: Hạn chế cũ là suy đoán.</t>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="2" shapeId="0">
+      <text>
+        <t>[Lần 5] Giá trị trước:
+Tác giả nêu (tr. 19): lead time cố định, RL tốn kém, DRL/DL khó diễn giải. Nhận định nhóm: không phải toàn bộ M5, không có thanh lý, không phân tích ADI–CV²
+Lý do: Làm rõ các nhận định phủ định bằng kết quả tìm từ khóa trong PDF.</t>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="2" shapeId="0">
+      <text>
+        <t>[Lần 5] Giá trị trước:
+8.000 chuỗi bán nhiều của M5, 58 đặc trưng, train/test 75:25 (tr. 4)
+Lý do: Sửa trang trích: '58 đặc trưng' nằm trong abstract.</t>
+      </text>
+    </comment>
+    <comment ref="F23" authorId="2" shapeId="0">
+      <text>
+        <t>[Lần 5] Giá trị trước:
+Tác giả nêu: không đánh giá chuỗi bán thưa/chậm (tr. 4); tốn tính toán (45–60 phút GPU); GARCH giả định phần dư dừng; chỉ dùng M5 (tr. 16–17). Không báo cáo KPI tồn kho
+Lý do: SAI trước đó: 'Không báo cáo KPI tồn kho'. Bài có phép tính chi phí tồn kho kỳ vọng ở tr. 15.</t>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="2" shapeId="0">
+      <text>
+        <t>[Lần 5] Giá trị trước:
+Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không có KPI tồn kho; phải loại kỳ bằng 0 khỏi MAPE (abstract)
+Lý do: SAI trước đó: 'không có KPI tồn kho'. Bài có phân tích tồn kho dư ở tr. 7.</t>
       </text>
     </comment>
   </commentList>
@@ -1139,7 +1172,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Nhận định nhóm: không đánh giá việc dùng phân vị cho quyết định tồn kho</t>
+          <t>Tác giả nêu: M5 không tập trung vào một bài toán ra quyết định cụ thể và không định nghĩa tham số của bài toán đó (tr. 2–3). Phân vị cao 0,925–0,995 thường dùng để xác định safety stock (tr. 2)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2289,9 +2322,9 @@
           <t>Tập con thực phẩm biến động mạnh của M5 (tr. 8); môi trường RL từ dữ liệu thực + tổng hợp; mô phỏng 365 ngày (tr. 8)</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Tác giả nêu (tr. 19): lead time cố định, RL tốn kém, DRL/DL khó diễn giải. Nhận định nhóm: không phải toàn bộ M5, không có thanh lý, không phân tích ADI–CV²</t>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Tác giả nêu (tr. 19): lead time cố định, RL tốn kém, DRL/DL khó diễn giải. Nhận định nhóm: chỉ tập con thực phẩm (tr. 8); không có quyết định thanh lý (không có từ khóa liên quan); không phân loại ADI–CV² (chỉ nhắc định tính hàng bán chậm, tr. 16); dùng MAPE (tr. 6)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2348,14 +2381,14 @@
           <t>Stacked ensemble XGBoost + LightGBM + LSTM-GRU, GARCH(1,1) cho phương sai có điều kiện (tr. 6–8)</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>8.000 chuỗi bán nhiều của M5, 58 đặc trưng, train/test 75:25 (tr. 4)</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Tác giả nêu: không đánh giá chuỗi bán thưa/chậm (tr. 4); tốn tính toán (45–60 phút GPU); GARCH giả định phần dư dừng; chỉ dùng M5 (tr. 16–17). Không báo cáo KPI tồn kho</t>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>8.000 chuỗi bán nhiều của M5 (Bảng 2, tr. 4); 58 đặc trưng (abstract); train/test 75:25 (tr. 4)</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Tác giả nêu: không đánh giá chuỗi thưa/chậm, là 'điểm yếu chính' (tr. 4, 18); tốn tính toán, GARCH giả định dừng, chỉ M5 (tr. 16–17). Kết quả tồn kho chỉ có 1 phép tính minh họa: safety stock theo GARCH giảm chi phí kỳ vọng 11,8% (tr. 15)</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -2545,9 +2578,9 @@
           <t>Dữ liệu mua/sử dụng phụ tùng 2020–2024 của một nhà máy, theo tháng, chọn mặt hàng có chủ đích (tr. 2)</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không có KPI tồn kho; phải loại kỳ bằng 0 khỏi MAPE (abstract)</t>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không mô phỏng chính sách. Bài có ghi nhận tồn cuối kỳ vượt xa safety stock và ước tính tiết kiệm ~2,6 tỷ IDR chi phí lưu kho/năm (tr. 7); loại kỳ bằng 0 khỏi MAPE (abstract)</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -2650,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4824,6 +4857,138 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>LẦN 5 (29/09/2026): rà soát bằng PDF các bài 01–03, 21–25</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Nhận định nhóm: không đánh giá việc dùng phân vị cho quyết định tồn kho</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Tác giả nêu: M5 không tập trung vào một bài toán ra quyết định cụ thể và không định nghĩa tham số của bài toán đó (tr. 2–3). Phân vị cao 0,925–0,995 thường dùng để xác định safety stock (tr. 2)</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 5] Thay nhận định nhóm bằng câu có trong bài (PDF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Tác giả nêu (tr. 19): lead time cố định, RL tốn kém, DRL/DL khó diễn giải. Nhận định nhóm: không phải toàn bộ M5, không có thanh lý, không phân tích ADI–CV²</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>Tác giả nêu (tr. 19): lead time cố định, RL tốn kém, DRL/DL khó diễn giải. Nhận định nhóm: chỉ tập con thực phẩm (tr. 8); không có quyết định thanh lý (không có từ khóa liên quan); không phân loại ADI–CV² (chỉ nhắc định tính hàng bán chậm, tr. 16); dùng MAPE (tr. 6)</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 5] Làm rõ các nhận định phủ định bằng kết quả tìm từ khóa trong PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Dataset ở đâu</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>8.000 chuỗi bán nhiều của M5, 58 đặc trưng, train/test 75:25 (tr. 4)</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>8.000 chuỗi bán nhiều của M5 (Bảng 2, tr. 4); 58 đặc trưng (abstract); train/test 75:25 (tr. 4)</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 5] Sửa trang trích: '58 đặc trưng' nằm trong abstract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Tác giả nêu: không đánh giá chuỗi bán thưa/chậm (tr. 4); tốn tính toán (45–60 phút GPU); GARCH giả định phần dư dừng; chỉ dùng M5 (tr. 16–17). Không báo cáo KPI tồn kho</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Tác giả nêu: không đánh giá chuỗi thưa/chậm, là 'điểm yếu chính' (tr. 4, 18); tốn tính toán, GARCH giả định dừng, chỉ M5 (tr. 16–17). Kết quả tồn kho chỉ có 1 phép tính minh họa: safety stock theo GARCH giảm chi phí kỳ vọng 11,8% (tr. 15)</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 5] SAI trước đó: 'Không báo cáo KPI tồn kho'. Bài có phép tính chi phí tồn kho kỳ vọng ở tr. 15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không có KPI tồn kho; phải loại kỳ bằng 0 khỏi MAPE (abstract)</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Nhận định nhóm: dữ liệu nhỏ, một nhà máy, không phải bán lẻ; không mô phỏng chính sách. Bài có ghi nhận tồn cuối kỳ vượt xa safety stock và ước tính tiết kiệm ~2,6 tỷ IDR chi phí lưu kho/năm (tr. 7); loại kỳ bằng 0 khỏi MAPE (abstract)</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 5] SAI trước đó: 'không có KPI tồn kho'. Bài có phân tích tồn kho dư ở tr. 7.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
review: add secondary source for paper 20; reject Logistics 9(3):126 as substitute
</commit_message>
<xml_diff>
--- a/M5_papers_baseline_gap.xlsx
+++ b/M5_papers_baseline_gap.xlsx
@@ -98,7 +98,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -148,6 +148,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -233,6 +236,7 @@
     <author>Claude (lần 5 – rà soát bằng PDF)</author>
     <author>Claude (rà soát 29/09/2026 – lần 2)</author>
     <author>Claude (lần 4)</author>
+    <author>Claude (lần 6)</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0">
@@ -610,6 +614,13 @@
         <t>[Lần 2] Giá trị trước:
 Chỉ xét mô hình thống kê (họ exponential smoothing), chưa xét mô hình ML toàn cục
 Lý do sửa: Hạn chế cũ là suy đoán.</t>
+      </text>
+    </comment>
+    <comment ref="F21" authorId="5" shapeId="0">
+      <text>
+        <t>[Lần 6] Giá trị trước:
+[Chưa kiểm chứng]
+Lý do: bổ sung nguồn thứ cấp đọc được.</t>
       </text>
     </comment>
     <comment ref="F22" authorId="2" shapeId="0">
@@ -2258,9 +2269,9 @@
           <t>[Chưa kiểm chứng] Theo tên bài: dữ liệu M5</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
-        <is>
-          <t>[Chưa kiểm chứng]</t>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>[Chưa đọc được bài] Nguồn thứ cấp: Tichy et al. (2025, J. Forecasting; arXiv 2211.16313 tr. 3) trích bài này để ủng hộ ý 'chất lượng dự báo chỉ là phương tiện cho quyết định, có thể trở nên không quan trọng'. Không phải kết quả trực tiếp của bài 20</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
@@ -2683,7 +2694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4989,6 +5000,65 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="19" t="inlineStr">
+        <is>
+          <t>LẦN 6 (29/09/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>[Chưa kiểm chứng]</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>[Chưa đọc được bài] Nguồn thứ cấp: Tichy et al. (2025, J. Forecasting; arXiv 2211.16313 tr. 3) trích bài này để ủng hộ ý 'chất lượng dự báo chỉ là phương tiện cho quyết định, có thể trở nên không quan trọng'. Không phải kết quả trực tiếp của bài 20</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 6] Bổ sung nguồn thứ cấp (Tichy et al., 2025) cho bài 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>(loại)</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>logistics-09-00126.pdf</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Leveraging Household Food Waste Consumer Behaviour to Optimise Logistics (Ntai et al., 2025, Logistics 9(3):126)</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>KHÔNG đưa vào / không thay thế bài 20: khảo sát ~200 hộ gia đình, hồi quy, không có dự báo, không dùng M5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
review: add user-provided summary of paper 19 (Kourentzes 2020), marked unverified
</commit_message>
<xml_diff>
--- a/M5_papers_baseline_gap.xlsx
+++ b/M5_papers_baseline_gap.xlsx
@@ -236,6 +236,7 @@
     <author>Claude (lần 5 – rà soát bằng PDF)</author>
     <author>Claude (rà soát 29/09/2026 – lần 2)</author>
     <author>Claude (lần 4)</author>
+    <author>Claude (lần 7)</author>
     <author>Claude (lần 6)</author>
   </authors>
   <commentList>
@@ -595,28 +596,40 @@
 Lý do: Bổ sung nguồn.</t>
       </text>
     </comment>
-    <comment ref="D20" authorId="3" shapeId="0">
+    <comment ref="D20" authorId="5" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Tối ưu / chọn mô hình dự báo theo tiêu chí gắn với tồn kho thay vì chỉ sai số dự báo
-Lý do sửa: Toàn văn chưa tải được; 'họ exponential smoothing' chưa kiểm chứng.</t>
+Lý do sửa: Toàn văn chưa tải được; 'họ exponential smoothing' chưa kiểm chứng.
+---
+[Lần 7] Giá trị trước:
+Tối ưu tham số mô hình dự báo bằng cách đưa trực tiếp metric và chính sách tồn kho vào hàm mục tiêu (trang mô tả kho Lancaster). [Chưa kiểm chứng: họ mô hình cụ thể]
+Lý do: bổ sung từ tóm tắt người dùng cung cấp (chưa đối chiếu PDF).</t>
       </text>
     </comment>
-    <comment ref="E20" authorId="3" shapeId="0">
+    <comment ref="E20" authorId="5" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Dữ liệu bán lẻ và mô phỏng
-Lý do sửa: SAI trước đó: 'bán lẻ và mô phỏng' chưa kiểm chứng.</t>
+Lý do sửa: SAI trước đó: 'bán lẻ và mô phỏng' chưa kiểm chứng.
+---
+[Lần 7] Giá trị trước:
+Dữ liệu thực (trang mô tả kho Lancaster). [Chưa kiểm chứng: số chuỗi, ngành]
+Lý do: bổ sung từ tóm tắt người dùng cung cấp (chưa đối chiếu PDF).</t>
       </text>
     </comment>
-    <comment ref="F20" authorId="3" shapeId="0">
+    <comment ref="F20" authorId="5" shapeId="0">
       <text>
         <t>[Lần 2] Giá trị trước:
 Chỉ xét mô hình thống kê (họ exponential smoothing), chưa xét mô hình ML toàn cục
-Lý do sửa: Hạn chế cũ là suy đoán.</t>
+Lý do sửa: Hạn chế cũ là suy đoán.
+---
+[Lần 7] Giá trị trước:
+[Chưa kiểm chứng — cần mở toàn văn]
+Lý do: bổ sung từ tóm tắt người dùng cung cấp (chưa đối chiếu PDF).</t>
       </text>
     </comment>
-    <comment ref="F21" authorId="5" shapeId="0">
+    <comment ref="F21" authorId="6" shapeId="0">
       <text>
         <t>[Lần 6] Giá trị trước:
 [Chưa kiểm chứng]
@@ -2197,17 +2210,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu tham số mô hình dự báo bằng cách đưa trực tiếp metric và chính sách tồn kho vào hàm mục tiêu (trang mô tả kho Lancaster). [Chưa kiểm chứng: họ mô hình cụ thể]</t>
+          <t>Tối ưu tham số dự báo bằng cách đưa metric và chính sách tồn kho vào hàm mục tiêu (trang mô tả Lancaster). [Theo tóm tắt người dùng — chưa đối chiếu PDF] Vòng mô phỏng tồn kho: dự báo → mô phỏng → KPI → chỉnh tham số</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Dữ liệu thực (trang mô tả kho Lancaster). [Chưa kiểm chứng: số chuỗi, ngành]</t>
+          <t>Dữ liệu thực (trang mô tả Lancaster). [Theo tóm tắt người dùng — chưa đối chiếu PDF] 229 SKU hàng tiêu dùng của một nhà sản xuất ở Anh, theo tuần, 173 quan sát/SKU, lead time 3–5 tuần</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>[Chưa kiểm chứng — cần mở toàn văn]</t>
+          <t>[Theo tóm tắt người dùng — chưa đối chiếu PDF] Dự báo tối ưu theo tồn kho kém chính xác hơn (tới ~9%) nhưng bias ngoài mẫu cải thiện tới ~62%; mô hình MSE nhỏ nhất không phải mô hình chi phí tồn kho nhỏ nhất. Hạn chế do tác giả nêu: chưa kiểm chứng</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -2240,7 +2253,7 @@
       </c>
       <c r="M20" s="8" t="inlineStr">
         <is>
-          <t>[Nội dung] Chỉ đọc trang mô tả kho Lancaster — 29/09/2026
+          <t>[Nội dung] Chỉ đọc trang mô tả kho Lancaster — 29/09/2026 + tóm tắt người dùng (chưa đối chiếu)
 [Metadata] ✅ Crossref khớp tên/tác giả/tạp chí/trang; DOI chuyển đúng nhà xuất bản</t>
         </is>
       </c>
@@ -2694,7 +2707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5059,6 +5072,88 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>LẦN 7 (29/09/2026): tóm tắt bài 19 do người dùng cung cấp</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Model đã dùng</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>Tối ưu tham số mô hình dự báo bằng cách đưa trực tiếp metric và chính sách tồn kho vào hàm mục tiêu (trang mô tả kho Lancaster). [Chưa kiểm chứng: họ mô hình cụ thể]</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Tối ưu tham số dự báo bằng cách đưa metric và chính sách tồn kho vào hàm mục tiêu (trang mô tả Lancaster). [Theo tóm tắt người dùng — chưa đối chiếu PDF] Vòng mô phỏng tồn kho: dự báo → mô phỏng → KPI → chỉnh tham số</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 7] Bổ sung từ tóm tắt người dùng; chưa đối chiếu PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Dataset ở đâu</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu thực (trang mô tả kho Lancaster). [Chưa kiểm chứng: số chuỗi, ngành]</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu thực (trang mô tả Lancaster). [Theo tóm tắt người dùng — chưa đối chiếu PDF] 229 SKU hàng tiêu dùng của một nhà sản xuất ở Anh, theo tuần, 173 quan sát/SKU, lead time 3–5 tuần</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 7] Bổ sung từ tóm tắt người dùng; chưa đối chiếu PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>Limit (hạn chế)</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>[Chưa kiểm chứng — cần mở toàn văn]</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>[Theo tóm tắt người dùng — chưa đối chiếu PDF] Dự báo tối ưu theo tồn kho kém chính xác hơn (tới ~9%) nhưng bias ngoài mẫu cải thiện tới ~62%; mô hình MSE nhỏ nhất không phải mô hình chi phí tồn kho nhỏ nhất. Hạn chế do tác giả nêu: chưa kiểm chứng</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 7] Bổ sung từ tóm tắt người dùng; chưa đối chiếu PDF</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
review: move paper 20 (Theodorou 2025) to watch-list; steps 3-4 no longer rely on it
</commit_message>
<xml_diff>
--- a/M5_papers_baseline_gap.xlsx
+++ b/M5_papers_baseline_gap.xlsx
@@ -238,6 +238,7 @@
     <author>Claude (lần 4)</author>
     <author>Claude (lần 7)</author>
     <author>Claude (lần 6)</author>
+    <author>Claude (lần 8)</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0">
@@ -634,6 +635,20 @@
         <t>[Lần 6] Giá trị trước:
 [Chưa kiểm chứng]
 Lý do: bổ sung nguồn thứ cấp đọc được.</t>
+      </text>
+    </comment>
+    <comment ref="K21" authorId="7" shapeId="0">
+      <text>
+        <t>[Lần 8] Giá trị trước:
+Domain (inventory) + M5
+Lý do: không tải được PDF; nhóm quyết định không dùng bài 20 làm căn cứ.</t>
+      </text>
+    </comment>
+    <comment ref="L21" authorId="7" shapeId="0">
+      <text>
+        <t>[Lần 8] Giá trị trước:
+★★★ (có thể trùng hướng — BẮT BUỘC đọc)
+Lý do: không tải được PDF; nhóm quyết định không dùng bài 20 làm căn cứ.</t>
       </text>
     </comment>
     <comment ref="F22" authorId="2" shapeId="0">
@@ -2307,12 +2322,12 @@
       </c>
       <c r="K21" s="15" t="inlineStr">
         <is>
-          <t>Domain (inventory) + M5</t>
+          <t>Ngoài danh sách chính thức</t>
         </is>
       </c>
       <c r="L21" s="15" t="inlineStr">
         <is>
-          <t>★★★ (có thể trùng hướng — BẮT BUỘC đọc)</t>
+          <t>⛔ Theo dõi — KHÔNG dùng làm căn cứ (không truy cập được toàn văn)</t>
         </is>
       </c>
       <c r="M21" s="15" t="inlineStr">
@@ -2707,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2768,7 +2783,7 @@
       <c r="A6" s="17" t="inlineStr"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Dòng bài chưa đọc được nội dung (bài 20) — không được dùng nội dung cho tới khi có PDF</t>
+          <t>Dòng bài 20 — không đọc được toàn văn; nằm ngoài danh sách chính thức, KHÔNG dùng làm căn cứ</t>
         </is>
       </c>
     </row>
@@ -5151,6 +5166,63 @@
       <c r="E115" s="3" t="inlineStr">
         <is>
           <t>[Lần 7] Bổ sung từ tóm tắt người dùng; chưa đối chiếu PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>LẦN 8 (29/09/2026): bài 20 chuyển sang 'theo dõi', không dùng làm căn cứ</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Mức liên quan</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>★★★ (có thể trùng hướng — BẮT BUỘC đọc)</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>⛔ Theo dõi — KHÔNG dùng làm căn cứ (không truy cập được toàn văn)</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 8] Chuyển bài 20 sang danh sách theo dõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Nhóm bài (README Bước 2)</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Domain (inventory) + M5</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>Ngoài danh sách chính thức</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>[Lần 8] Chuyển bài 20 sang danh sách theo dõi</t>
         </is>
       </c>
     </row>

</xml_diff>